<commit_message>
redesign(home): kompaktere Module, radiale Slabs, About-Umbau
- Use-Case: Zeilen kompakter + rechts angedockt (links mehr Luft); Bildcontainer
  full-bleed (Screen-zu-Screen) mit radialen Kanten.
- About-Slab: Supertools-Logo raus, Eyebrow nach oben, Headline hochgezogen
  (bündig mit den Prinzip-Linien rechts); die beiden CTAs (Behörden/Anbieter)
  kompakt in die rechte Lücke unter die Prinzipien gesetzt.
- Redaktionelle Schwerpunkte: als ein radialer Stone-Slab gerahmt (weiche
  Kanten zur Cream-Fläche), Abstand Feature↔Cluster reduziert. Schwarze Linie
  über die volle Gridbreite. Cluster-Cover kleiner + abgerundet, Eyebrow als
  Chip über dem Bild, Artikel als modulare weiße Karten.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Amtshelden_Zielkundenliste_Sponsoring_2026 (1).xlsx
+++ b/Amtshelden_Zielkundenliste_Sponsoring_2026 (1).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wolfram/web-projekte/supertools/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B5E7897B-ACE0-F946-98B7-A1CD209FD6AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3C0FF1A4-9A0E-DF44-9D90-1F5E32751745}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="27000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>